<commit_message>
fix(inventory): apply one source-specific Li-O2 recycling route
Use Wang et al. (2020), DOI 10.1016/j.jclepro.2020.121339, SI Table S16 per-kg recycling basis. Disable the internal -1/321 fragment with a zero formula/cache and route the full capacity-market waste mass to the existing RER LiO2 recycling activity. Retain treatment recipes, production and disposal mass/bounds, energy density and lifetime. The zero row can remain in DefaultInventory. Standalone manufacture becomes manufacturing-only; historical recovery performance and system mass basis are not validated. No new recovery credits or primary/secondary shares.

Scope: existing supplemental workbook inventories only. Approved as item 1 of ten on 2026-10-18.

Validation: exact edited-cell/ZIP-part scope, formula/cache round-trip and raw no-write ExcelImporter regression. Shared ecoinvent 3.8-3.12 checks are run after the batch; this does not constitute a full scenario rebuild.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-batteries-LiO2.xlsx
+++ b/premise/data/additional_inventories/lci-batteries-LiO2.xlsx
@@ -5231,8 +5231,12 @@
       <c r="A269" t="s">
         <v>3</v>
       </c>
-      <c r="B269" t="s">
-        <v>279</v>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>APPROVED Li-O2 SINGLE RECYCLING BOUNDARY, 2026-10-18. Wang, Deng and Yuan (2020), DOI 10.1016/j.jclepro.2020.121339, supporting information Table S16, explicitly describes recycling per 1 kg Li-O2 battery system. Its six treatment coefficients are retained. Set the former -1/321 kg/kg internal treatment fragment to a deterministic zero and apply end of life only at market for battery capacity, Li-ion, Li-O2: the full purchased battery mass is sent to treatment of LiO2 battery, for recycling (RER; waste LiO2 battery). Standalone manufacture is manufacturing-only. DefaultInventory may retain the zero exchange; it contributes no treatment flow. Do not add a second generic Li-ion route. This restores a single historical source-specific accounting route; treatment yields, whole-system mass normalization, modern recovery and primary/secondary shares remain unvalidated. No new recovery credit or change to manufacturing recipes, density or lifetime.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+System: 63.5kWh Li-O2 || Mass (excl. O2 tanks): 267 kg || Battery energy density: 238 Wh/kg || System energy density (incl. O2 tanks): 198 Wh/kg || Battery lifetime: 305 kWh/kg (1.76 MJ/km x 2e5 km / 321 kg). Source: Originally from Wang, F., Deng, Y., &amp; Yuan, C. (2020). Life cycle assessment of lithium oxygen battery for electric vehicles. Journal of Cleaner Production, 264, 121339. https://doi.org/10.1016/j.jclepro.2020.121339</t>
+        </is>
       </c>
     </row>
     <row r="270" spans="1:8" x14ac:dyDescent="0.2">
@@ -5471,8 +5475,8 @@
         <v>147</v>
       </c>
       <c r="B284">
-        <f>-1/321</f>
-        <v>-3.1152647975077881E-3</v>
+        <f>0</f>
+        <v>0</v>
       </c>
       <c r="C284" t="s">
         <v>9</v>
@@ -5485,6 +5489,11 @@
       </c>
       <c r="G284" t="s">
         <v>148</v>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Disabled duplicate treatment fragment: original formula -1/321 kg waste/kg battery; now zero. The capacity market applies the complete mass through the existing LiO2-specific recycling activity. See activity comment for source and limits.</t>
+        </is>
       </c>
     </row>
     <row r="286" spans="1:8" ht="16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
fix(inventory): restore Li-O2 collector facility input
Restore Wang et al. (2020), DOI 10.1016/j.jclepro.2020.121339, SI Table S10 aluminium casting-plant proxy: 1.5e-10 RER units/kg collector. Reuse an existing blank exchange row and existing supplier. Preserve aluminium feed, rolling and transport; the full manufacturing mass/yield balance remains unresolved.

Scope: existing supplemental workbook inventories only. Approved as item 3 of ten on 2026-10-18.

Validation: exact edited-cell/ZIP-part scope, formula/cache round-trip and raw no-write ExcelImporter regression. Shared ecoinvent 3.8-3.12 checks are run after the batch; this does not constitute a full scenario rebuild.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-batteries-LiO2.xlsx
+++ b/premise/data/additional_inventories/lci-batteries-LiO2.xlsx
@@ -3124,8 +3124,12 @@
       <c r="A134" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B134" s="7" t="s">
-        <v>263</v>
+      <c r="B134" s="7" t="inlineStr">
+        <is>
+          <t>APPROVED Li-O2 COLLECTOR FACILITY SOURCE OMISSION, 2026-10-18. Wang et al. (2020), DOI 10.1016/j.jclepro.2020.121339, supporting information Table S10 lists 1.5E-10 pieces RER aluminium casting plant per kg aluminium current collector. Add the existing RER aluminium casting facility construction supplier at 1.5E-10 unit/kg in blank exchange row 147. This restores the source infrastructure proxy; it does not validate the casting/rolling facility design, manufacturing yield or the unresolved 0.825 kg aluminium feed per kg output. Keep aluminium feed, sheet rolling, transport and all other coefficients unchanged.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+ Source: Originally from Wang, F., Deng, Y., &amp; Yuan, C. (2020). Life cycle assessment of lithium oxygen battery for electric vehicles. Journal of Cleaner Production, 264, 121339. https://doi.org/10.1016/j.jclepro.2020.121339</t>
+        </is>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.2">
@@ -3307,6 +3311,41 @@
       </c>
       <c r="G146" t="s">
         <v>91</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>aluminium casting facility construction</t>
+        </is>
+      </c>
+      <c r="B147">
+        <v>1.5e-10</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>RER</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>technosphere</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>aluminium casting facility</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Wang et al. (2020), DOI 10.1016/j.jclepro.2020.121339, SI Table S10: 1.5E-10 RER aluminium casting plant units/kg collector. Source facility proxy; no measured design or manufacturing-yield validation.</t>
+        </is>
       </c>
     </row>
     <row r="149" spans="1:8" ht="16" x14ac:dyDescent="0.2">

</xml_diff>